<commit_message>
feat: profitability model and dq report
- add pricing_plan rate card; settlement.fee_amount is now merchant revenue,
  route_cost remains provider cost, so contribution is derivable
- task 3: add PASS/FAIL result, reconciliation breakdown (zero residual),
  evidence samples for each failing blocking check
- task 4: star schema at one row per payment attempt, all one-to-many
  sources pre-aggregated to transaction grain before joining
- validation: transaction-side vs settlement-side reconcile at $566,298.30;
  naive joins shown to inflate 11.9x and 1.002x
</commit_message>
<xml_diff>
--- a/03_dq_report/03_dq_report.xlsx
+++ b/03_dq_report/03_dq_report.xlsx
@@ -16,6 +16,8 @@
     <sheet name="Settlement coverage by month" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Latency by provider month" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Fan-out proof" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Reconciliation breakdown" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Evidence samples" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +26,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="8">
     <font>
       <name val="Calibri"/>
@@ -90,12 +94,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
   </fills>
@@ -125,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,10 +144,19 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -511,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B14"/>
+  <dimension ref="B2:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -555,45 +568,2206 @@
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Severity</t>
+          <t>Severity vs result</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Blocking - corrupts the executive KPI if left untreated.</t>
+          <t>Severity is the potential impact of a check. Result is what happened when it ran.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Warning - biases a breakdown but not the headline number.</t>
+          <t>A Blocking check with result PASS is a control that held, not an open issue.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Informational - a valid business state, recorded so it is not mistaken for a defect.</t>
-        </is>
-      </c>
+      <c r="B11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="B12" s="3" t="inlineStr"/>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Remediation options</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Remediation options</t>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Exclude, repair, quarantine, or retain with a flag.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Exclude, repair, quarantine, or retain with a flag.</t>
+      <c r="B14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>The USD settlement mismatch decomposes to a zero residual. See the breakdown sheet.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Settlement rows that do not reconcile to transaction value in USD</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>3038</v>
+      </c>
+      <c r="C2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  explained by: transaction has two settlement rows (partial + correction)</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>2668</v>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Defect 'more than one settlement row per transaction'</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  explained by: transaction carries an impossible negative amount</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>370</v>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Defect 'amount &lt; 0 with status CAPTURED'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  unexplained residual</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Zero residual means the break is fully attributed to known defects</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>check_name</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>columns_shown</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>col_1</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>col_2</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>col_3</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>col_4</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>col_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>transaction.amount &lt; 0 with status CAPTURED (impossible)</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, status</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000785</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>MER00540</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>-90.83</v>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>transaction.amount &lt; 0 with status CAPTURED (impossible)</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, status</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>TXN00002071</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>MER00323</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>-3444.78</v>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>transaction.amount &lt; 0 with status CAPTURED (impossible)</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, status</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>TXN00002892</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>MER00581</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>-60.95</v>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>SGD</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>transaction.amount &lt; 0 with status CAPTURED (impossible)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, status</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>TXN00003008</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>MER00069</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>-14347.75</v>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>transaction.amount &lt; 0 with status CAPTURED (impossible)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, status</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>TXN00003601</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v/>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>-2234.38</v>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>transaction.amount &lt; 0 with status CAPTURED (impossible)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, status</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>TXN00005162</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>MER00323</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>-3346.85</v>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>transaction.amount &lt; 0 with status CAPTURED (impossible)</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, status</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>TXN00005967</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>MER00241</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>-324.83</v>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>transaction.amount &lt; 0 with status CAPTURED (impossible)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, status</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>TXN00006000</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>MER00284</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>-11.13</v>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>transaction.amount &lt; 0 with status CAPTURED (impossible)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, status</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>TXN00006554</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>MER00458</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>-9.789999999999999</v>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>SGD</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>transaction.amount &lt; 0 with status CAPTURED (impossible)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, status</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>TXN00008056</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>MER00431</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>-713.37</v>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>fraud_decision.risk_score outside 0 to 1</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, rule_id, decision, risk_score, model_version</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>TXN00156327</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>FR_VELOCITY</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>APPROVE</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>51.94</v>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>v3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>fraud_decision.risk_score outside 0 to 1</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, rule_id, decision, risk_score, model_version</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>TXN00156327</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>FR_AMOUNT</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>APPROVE</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>38.79</v>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>v3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>fraud_decision.risk_score outside 0 to 1</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, rule_id, decision, risk_score, model_version</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>TXN00156327</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>FR_GEO</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>APPROVE</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>32.71</v>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>v3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>fraud_decision.risk_score outside 0 to 1</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, rule_id, decision, risk_score, model_version</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>TXN00156327</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>FR_GEO</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>APPROVE</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>45.58</v>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>v3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>fraud_decision.risk_score outside 0 to 1</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, rule_id, decision, risk_score, model_version</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>TXN00156328</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>FR_GEO</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>APPROVE</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>32.63</v>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>v3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>fraud_decision.risk_score outside 0 to 1</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, rule_id, decision, risk_score, model_version</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>TXN00156330</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>FR_AMOUNT</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>APPROVE</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>v3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>fraud_decision.risk_score outside 0 to 1</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, rule_id, decision, risk_score, model_version</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>TXN00156330</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>FR_DEVICE</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>APPROVE</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>20.27</v>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>v3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>fraud_decision.risk_score outside 0 to 1</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, rule_id, decision, risk_score, model_version</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>TXN00156331</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>FR_DEVICE</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>APPROVE</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>54.04</v>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>v3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>fraud_decision.risk_score outside 0 to 1</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, rule_id, decision, risk_score, model_version</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>TXN00156331</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>FR_GEO</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>APPROVE</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>19.65</v>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>v3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>fraud_decision.risk_score outside 0 to 1</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, rule_id, decision, risk_score, model_version</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>TXN00156331</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>FR_DEVICE</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>APPROVE</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>44.32</v>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>v3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>more than one settlement row per transaction</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000008</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>2060.87</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>29.3281</v>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>more than one settlement row per transaction</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000008</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>2669.45</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>37.9889</v>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>CORRECTION</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>more than one settlement row per transaction</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000146</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>374.45</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>5.3984</v>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>more than one settlement row per transaction</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000146</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>323.23</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>CORRECTION</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>more than one settlement row per transaction</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000468</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>68.15000000000001</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>1.4913</v>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>CORRECTION</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>more than one settlement row per transaction</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000468</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>70.26000000000001</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>1.5374</v>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>more than one settlement row per transaction</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000606</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>18.03</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>0.4547</v>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>CORRECTION</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>more than one settlement row per transaction</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000606</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>24.35</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>0.6142</v>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>more than one settlement row per transaction</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000736</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>23.36</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>0.4231</v>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>more than one settlement row per transaction</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000736</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>42.56</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>0.7707000000000001</v>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>CORRECTION</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>settlement.transaction_id not found in transaction</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>TXN90000301</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>23.44</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>0.6824</v>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>settlement.transaction_id not found in transaction</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>TXN90000237</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>90.56</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>2.0523</v>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>settlement.transaction_id not found in transaction</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>TXN90000267</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>972.12</v>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>15.9288</v>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>settlement.transaction_id not found in transaction</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>TXN90000279</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>182.16</v>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>2.107</v>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>settlement.transaction_id not found in transaction</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>TXN90000332</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>144.2</v>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>2.146</v>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>CORRECTION</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>settlement.transaction_id not found in transaction</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>TXN90000213</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>44.55</v>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>1.1132</v>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>settlement.transaction_id not found in transaction</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>TXN90000066</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="n">
+        <v>21.41</v>
+      </c>
+      <c r="E38" s="6" t="n">
+        <v>0.6411</v>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>settlement.transaction_id not found in transaction</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>TXN90000056</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>245.65</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>3.6401</v>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>settlement.transaction_id not found in transaction</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>TXN90000187</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="n">
+        <v>567.88</v>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>6.3971</v>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>settlement.transaction_id not found in transaction</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, settlement_amount, fee_amount, settlement_status</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>TXN90000439</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="n">
+        <v>21.24</v>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>0.6375999999999999</v>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>captured transaction with no settlement row</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, created_at</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000002</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>MER00347</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="n">
+        <v>510.46</v>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="G42" s="12" t="n">
+        <v>45658.00683716113</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>captured transaction with no settlement row</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, created_at</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000053</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>MER00216</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>2250.94</v>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="G43" s="12" t="n">
+        <v>45658.11892730565</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>captured transaction with no settlement row</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, created_at</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000062</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>MER00273</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="n">
+        <v>6273.87</v>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="G44" s="12" t="n">
+        <v>45658.13598548505</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>captured transaction with no settlement row</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, created_at</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000064</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="n">
+        <v/>
+      </c>
+      <c r="E45" s="6" t="n">
+        <v>55244.81</v>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="G45" s="12" t="n">
+        <v>45658.13978467941</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>captured transaction with no settlement row</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, created_at</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000177</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>MER00323</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="n">
+        <v>4607.14</v>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="G46" s="12" t="n">
+        <v>45658.36039633919</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>captured transaction with no settlement row</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, created_at</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000212</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>MER00237</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="G47" s="12" t="n">
+        <v>45658.43647590835</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>captured transaction with no settlement row</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, created_at</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000240</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>MER00569</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="n">
+        <v>16549.18</v>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="G48" s="12" t="n">
+        <v>45658.48450988022</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>captured transaction with no settlement row</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, created_at</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000256</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>MER00373</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="n">
+        <v>2384.94</v>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="G49" s="12" t="n">
+        <v>45658.5108965728</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>captured transaction with no settlement row</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, created_at</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000408</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>MER00084</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="n">
+        <v>103399.19</v>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="G50" s="12" t="n">
+        <v>45658.78088128351</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>captured transaction with no settlement row</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, merchant_id, amount, currency, created_at</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000435</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>MER00362</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="n">
+        <v>92.7</v>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>SGD</t>
+        </is>
+      </c>
+      <c r="G51" s="12" t="n">
+        <v>45658.83437039357</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>transaction.merchant_id is null</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, customer_id, channel, amount, status</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000055</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>CUS003930</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
+        <v>11116.17</v>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>transaction.merchant_id is null</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, customer_id, channel, amount, status</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000064</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>CUS009466</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>WALLET</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
+        <v>55244.81</v>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>transaction.merchant_id is null</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, customer_id, channel, amount, status</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000204</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>CUS006714</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>CARD</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
+        <v>50.16</v>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>transaction.merchant_id is null</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, customer_id, channel, amount, status</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000344</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>CUS000473</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
+        <v>13407.63</v>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>transaction.merchant_id is null</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, customer_id, channel, amount, status</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000437</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>CUS012089</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>WALLET</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
+        <v>2990.36</v>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>DECLINED</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>transaction.merchant_id is null</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, customer_id, channel, amount, status</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>TXN00000672</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>CUS005413</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>WALLET</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
+        <v>280.87</v>
+      </c>
+      <c r="G57" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>transaction.merchant_id is null</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, customer_id, channel, amount, status</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>TXN00001032</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>CUS003047</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>WALLET</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n">
+        <v>10509.14</v>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>transaction.merchant_id is null</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, customer_id, channel, amount, status</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>TXN00001214</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>CUS012899</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>WALLET</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n">
+        <v>44825.26</v>
+      </c>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>transaction.merchant_id is null</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, customer_id, channel, amount, status</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>TXN00002101</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>CUS000386</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="n">
+        <v>24897.13</v>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>transaction.merchant_id is null</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>transaction_id, customer_id, channel, amount, status</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>TXN00002149</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>CUS009089</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>CARD</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>366.1</v>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
         </is>
       </c>
     </row>
@@ -608,7 +2782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -617,8 +2791,9 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -654,10 +2829,15 @@
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
           <t>severity</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>remediation</t>
         </is>
@@ -690,10 +2870,15 @@
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>Repair - normalise by model_version before any threshold comparison</t>
         </is>
@@ -726,10 +2911,15 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>Retain with flag and impute the fee from route_cost; excluding them biases recent months</t>
         </is>
@@ -762,10 +2952,15 @@
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>Sum settlement rows to transaction grain before reconciling</t>
         </is>
@@ -798,10 +2993,15 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>Sum fee_amount to transaction grain before joining</t>
         </is>
@@ -834,10 +3034,15 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>Exclude and report as a reconciliation break to Finance Operations</t>
         </is>
@@ -870,10 +3075,15 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>Quarantine - a captured payment cannot carry a negative amount</t>
         </is>
@@ -904,12 +3114,17 @@
       <c r="F8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>Quarantine - cannot compute value</t>
         </is>
@@ -940,12 +3155,17 @@
       <c r="F9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>Quarantine</t>
         </is>
@@ -976,12 +3196,17 @@
       <c r="F10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>Repair from source</t>
         </is>
@@ -1012,12 +3237,17 @@
       <c r="F11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Repair from source</t>
         </is>
@@ -1048,12 +3278,17 @@
       <c r="F12" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>Deduplicate - the declared primary key must hold</t>
         </is>
@@ -1084,12 +3319,17 @@
       <c r="F13" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>Deduplicate</t>
         </is>
@@ -1120,12 +3360,17 @@
       <c r="F14" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>Deduplicate</t>
         </is>
@@ -1156,12 +3401,17 @@
       <c r="F15" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>Quarantine - orphaned merchant reference</t>
         </is>
@@ -1192,12 +3442,17 @@
       <c r="F16" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>Exclude</t>
         </is>
@@ -1228,12 +3483,17 @@
       <c r="F17" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>Quarantine - a payment that never captured cannot be charged back</t>
         </is>
@@ -1264,12 +3524,17 @@
       <c r="F18" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>Quarantine - an event cannot precede its transaction</t>
         </is>
@@ -1300,12 +3565,17 @@
       <c r="F19" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>Quarantine</t>
         </is>
@@ -1336,12 +3606,17 @@
       <c r="F20" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>Quarantine</t>
         </is>
@@ -1372,12 +3647,17 @@
       <c r="F21" s="6" t="n">
         <v>4.437</v>
       </c>
-      <c r="G21" s="8" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
         <is>
           <t>Warning</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="I21" s="6" t="inlineStr">
         <is>
           <t>Retain - use event_time for KPI periods, ingestion_time for lag reporting</t>
         </is>
@@ -1408,12 +3688,17 @@
       <c r="F22" s="6" t="n">
         <v>0.679</v>
       </c>
-      <c r="G22" s="8" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
         <is>
           <t>Warning</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>Retain with flag; exclude only from merchant-level breakdowns</t>
         </is>
@@ -1444,12 +3729,17 @@
       <c r="F23" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G23" s="8" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
         <is>
           <t>Warning</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>Quarantine - zero-value attempts carry no economics</t>
         </is>
@@ -1480,12 +3770,17 @@
       <c r="F24" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G24" s="8" t="inlineStr">
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
         <is>
           <t>Warning</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="I24" s="6" t="inlineStr">
         <is>
           <t>Retain with flag - event pipeline gap</t>
         </is>
@@ -1516,12 +3811,17 @@
       <c r="F25" s="6" t="n">
         <v>21.914</v>
       </c>
-      <c r="G25" s="9" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H25" s="11" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>Retain - open cases are a valid business state</t>
         </is>
@@ -1552,12 +3852,17 @@
       <c r="F26" s="6" t="n">
         <v>0.75</v>
       </c>
-      <c r="G26" s="9" t="inlineStr">
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H26" s="11" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>Retain - genuine reversals, net them rather than dropping</t>
         </is>
@@ -1590,10 +3895,15 @@
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H27" s="11" t="inlineStr">
+        <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="I27" s="6" t="inlineStr">
         <is>
           <t>Retain</t>
         </is>
@@ -1615,7 +3925,7 @@
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -1632,7 +3942,7 @@
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>checks_failing</t>
+          <t>failing</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">

</xml_diff>